<commit_message>
Note expected COUNTIF values on Content Pillars tab
LibreOffice is non-functional in this environment (a one-formula test
workbook also times out), so the COUNTIF/SUM cells ship without cached
values and read blank outside Excel until first open. Results were
verified independently in Python: 3/2/3/2/2/2, total 14, matching the
14 calendar rows. The note records this for anyone previewing the file.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0159RBG9GE3t5Mafo8EcqW6e
</commit_message>
<xml_diff>
--- a/content/RK-World-LinkedIn-Content-Plan.xlsx
+++ b/content/RK-World-LinkedIn-Content-Plan.xlsx
@@ -1944,10 +1944,10 @@
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Weekly cadence</t>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Column F is a live COUNTIF against the Content Calendar tab, so it updates when you add or rename posts. Expected values: 3 / 2 / 3 / 2 / 2 / 2, total 14. Excel computes these on open; they may appear blank in a non-Excel previewer until then.</t>
         </is>
       </c>
     </row>
@@ -2045,8 +2045,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 15: listed everywhere vs available everywhere
New Category & market POV post on the gap between marketplace visibility
and real availability (out of stock, unserviceable pin code, wrong
fulfilment node). Added to both the markdown pack and the workbook, with
two new entries in the hook bank.

Pillar COUNTIF ranges on the Content Pillars tab widened to B5:B19;
counts re-verified in Python as 3/2/4/2/2/2, total 15.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0159RBG9GE3t5Mafo8EcqW6e
</commit_message>
<xml_diff>
--- a/content/RK-World-LinkedIn-Content-Plan.xlsx
+++ b/content/RK-World-LinkedIn-Content-Plan.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sources" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Content Calendar'!$A$4:$I$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Content Calendar'!$A$4:$I$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1206,15 +1206,63 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="46" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Category &amp; market POV</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Listed everywhere vs available everywhere</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Your brand is listed everywhere. But is it available everywhere?</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Opinion / 3-point breakdown</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Reach + inbound from brand teams</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Yellow = quotes financial figures sourced from third-party records; confirm internally before publishing.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I18"/>
+  <autoFilter ref="A4:I19"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -1229,7 +1277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1692,6 +1740,44 @@
       <c r="E17" s="5" t="inlineStr">
         <is>
           <t>#Milestone #Growth #Ecommerce #FMCG</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="338" customHeight="1">
+      <c r="A18" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Category &amp; market POV</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Listed everywhere vs available everywhere</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Your brand is listed everywhere.
+But is it available everywhere?
+Those aren't the same sentence. Most brands find that out the expensive way.
+A listing says your product exists. Availability says a customer in Siliguri can actually receive it - this week, at the price you set.
+Between those two facts sit three quiet failures:
+Listed, but out of stock. The page is live. The Buy Box isn't yours. A competitor's product just became the default answer to your brand name.
+Listed, but not serviceable. The customer finds you, enters their pin code, and the estimate reads seven days. They don't wait. They substitute.
+Listed, but in the wrong warehouse. Your inventory sits 1,800 km from the demand. Your ad spend created the intent. Someone else's supply chain captured it.
+None of these show up in a listing audit.
+All of them show up in your revenue.
+This is the whole reason we built the way we did - 125+ fulfilment centres, 19,000+ pin codes, 2,800+ brands.
+Not because scale is a vanity metric. Because available is a promise you can only keep by having inventory in the right place BEFORE the customer searches.
+Visibility gets you found.
+Availability gets you bought.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>#Ecommerce #FMCG #SupplyChain #Retail #BrandStrategy</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1870,7 @@
         </is>
       </c>
       <c r="F4" s="7">
-        <f>COUNTIF('Content Calendar'!$B$5:$B$18,B4)</f>
+        <f>COUNTIF('Content Calendar'!$B$5:$B$19,B4)</f>
         <v/>
       </c>
     </row>
@@ -1813,7 +1899,7 @@
         </is>
       </c>
       <c r="F5" s="8">
-        <f>COUNTIF('Content Calendar'!$B$5:$B$18,B5)</f>
+        <f>COUNTIF('Content Calendar'!$B$5:$B$19,B5)</f>
         <v/>
       </c>
     </row>
@@ -1842,7 +1928,7 @@
         </is>
       </c>
       <c r="F6" s="7">
-        <f>COUNTIF('Content Calendar'!$B$5:$B$18,B6)</f>
+        <f>COUNTIF('Content Calendar'!$B$5:$B$19,B6)</f>
         <v/>
       </c>
     </row>
@@ -1871,7 +1957,7 @@
         </is>
       </c>
       <c r="F7" s="8">
-        <f>COUNTIF('Content Calendar'!$B$5:$B$18,B7)</f>
+        <f>COUNTIF('Content Calendar'!$B$5:$B$19,B7)</f>
         <v/>
       </c>
     </row>
@@ -1900,7 +1986,7 @@
         </is>
       </c>
       <c r="F8" s="7">
-        <f>COUNTIF('Content Calendar'!$B$5:$B$18,B8)</f>
+        <f>COUNTIF('Content Calendar'!$B$5:$B$19,B8)</f>
         <v/>
       </c>
     </row>
@@ -1929,7 +2015,7 @@
         </is>
       </c>
       <c r="F9" s="8">
-        <f>COUNTIF('Content Calendar'!$B$5:$B$18,B9)</f>
+        <f>COUNTIF('Content Calendar'!$B$5:$B$19,B9)</f>
         <v/>
       </c>
     </row>
@@ -1947,7 +2033,7 @@
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Column F is a live COUNTIF against the Content Calendar tab, so it updates when you add or rename posts. Expected values: 3 / 2 / 3 / 2 / 2 / 2, total 14. Excel computes these on open; they may appear blank in a non-Excel previewer until then.</t>
+          <t>Column F is a live COUNTIF against the Content Calendar tab, so it updates when you add or rename posts. Expected values: 3 / 2 / 4 / 2 / 2 / 2, total 15. Excel computes these on open; they may appear blank in a non-Excel previewer until then.</t>
         </is>
       </c>
     </row>

</xml_diff>